<commit_message>
Make dense the canonical, reproducible submission pipeline
Clean re-measurement shows the dense (MiniLM + BM25 + TF-IDF) re-rank
finishes the 100K pool in ~180s on this laptop CPU — inside the 5-min
budget (the earlier 5m21s was inflated by the demo running alongside it).
So the dense ranking, which the approach deck already documents, is the
final submission.

- requirements.txt: restore sentence-transformers so rank.py reproduces
  the dense ranking (model committed under ./models, no download needed).
- Remove requirements-dense.txt (folded back in).
- README: dense enabled by default, ~180s; ~68s lexical fallback noted.
- submission_metadata.yaml: compute notes updated to ~180s dense.
- Submission artifacts (documents/*.csv/.xlsx, team_recruitertwin.csv)
  regenerated as the dense top-100 (rank1 1.030756 -> rank100 0.425364);
  passes validate_submission.py.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/amrutha.varma01_2783.xlsx
+++ b/documents/amrutha.varma01_2783.xlsx
@@ -40,16 +40,19 @@
     <t>CAND_0039754</t>
   </si>
   <si>
+    <t>CAND_0050454</t>
+  </si>
+  <si>
     <t>CAND_0046064</t>
   </si>
   <si>
-    <t>CAND_0050454</t>
+    <t>CAND_0044222</t>
   </si>
   <si>
     <t>CAND_0017960</t>
   </si>
   <si>
-    <t>CAND_0044222</t>
+    <t>CAND_0064326</t>
   </si>
   <si>
     <t>CAND_0011687</t>
@@ -58,21 +61,18 @@
     <t>CAND_0010685</t>
   </si>
   <si>
-    <t>CAND_0064326</t>
+    <t>CAND_0091534</t>
   </si>
   <si>
     <t>CAND_0068811</t>
   </si>
   <si>
+    <t>CAND_0043228</t>
+  </si>
+  <si>
     <t>CAND_0007009</t>
   </si>
   <si>
-    <t>CAND_0091534</t>
-  </si>
-  <si>
-    <t>CAND_0043228</t>
-  </si>
-  <si>
     <t>CAND_0088025</t>
   </si>
   <si>
@@ -82,12 +82,12 @@
     <t>CAND_0071974</t>
   </si>
   <si>
+    <t>CAND_0079387</t>
+  </si>
+  <si>
     <t>CAND_0008425</t>
   </si>
   <si>
-    <t>CAND_0079387</t>
-  </si>
-  <si>
     <t>CAND_0055905</t>
   </si>
   <si>
@@ -103,229 +103,229 @@
     <t>CAND_0005649</t>
   </si>
   <si>
+    <t>CAND_0083307</t>
+  </si>
+  <si>
+    <t>CAND_0070398</t>
+  </si>
+  <si>
+    <t>CAND_0069905</t>
+  </si>
+  <si>
+    <t>CAND_0028793</t>
+  </si>
+  <si>
+    <t>CAND_0061265</t>
+  </si>
+  <si>
+    <t>CAND_0075249</t>
+  </si>
+  <si>
     <t>CAND_0039383</t>
   </si>
   <si>
-    <t>CAND_0075249</t>
-  </si>
-  <si>
-    <t>CAND_0083307</t>
-  </si>
-  <si>
-    <t>CAND_0070398</t>
-  </si>
-  <si>
-    <t>CAND_0069905</t>
-  </si>
-  <si>
-    <t>CAND_0028793</t>
-  </si>
-  <si>
-    <t>CAND_0061265</t>
+    <t>CAND_0076251</t>
+  </si>
+  <si>
+    <t>CAND_0049896</t>
+  </si>
+  <si>
+    <t>CAND_0011432</t>
+  </si>
+  <si>
+    <t>CAND_0045250</t>
+  </si>
+  <si>
+    <t>CAND_0086151</t>
+  </si>
+  <si>
+    <t>CAND_0018549</t>
+  </si>
+  <si>
+    <t>CAND_0098846</t>
+  </si>
+  <si>
+    <t>CAND_0081852</t>
+  </si>
+  <si>
+    <t>CAND_0014440</t>
+  </si>
+  <si>
+    <t>CAND_0006567</t>
+  </si>
+  <si>
+    <t>CAND_0037566</t>
+  </si>
+  <si>
+    <t>CAND_0031593</t>
   </si>
   <si>
     <t>CAND_0027801</t>
   </si>
   <si>
-    <t>CAND_0011432</t>
-  </si>
-  <si>
-    <t>CAND_0086151</t>
-  </si>
-  <si>
-    <t>CAND_0049896</t>
-  </si>
-  <si>
-    <t>CAND_0076251</t>
-  </si>
-  <si>
-    <t>CAND_0018549</t>
-  </si>
-  <si>
-    <t>CAND_0045250</t>
-  </si>
-  <si>
     <t>CAND_0010257</t>
   </si>
   <si>
+    <t>CAND_0070485</t>
+  </si>
+  <si>
     <t>CAND_0016163</t>
   </si>
   <si>
-    <t>CAND_0098846</t>
-  </si>
-  <si>
-    <t>CAND_0081852</t>
-  </si>
-  <si>
-    <t>CAND_0006567</t>
-  </si>
-  <si>
-    <t>CAND_0037566</t>
-  </si>
-  <si>
-    <t>CAND_0014440</t>
-  </si>
-  <si>
-    <t>CAND_0031593</t>
-  </si>
-  <si>
-    <t>CAND_0070485</t>
+    <t>CAND_0053591</t>
   </si>
   <si>
     <t>CAND_0010770</t>
   </si>
   <si>
-    <t>CAND_0053591</t>
+    <t>CAND_0065878</t>
+  </si>
+  <si>
+    <t>CAND_0030953</t>
   </si>
   <si>
     <t>CAND_0093331</t>
   </si>
   <si>
-    <t>CAND_0065878</t>
-  </si>
-  <si>
-    <t>CAND_0030953</t>
+    <t>CAND_0095528</t>
+  </si>
+  <si>
+    <t>CAND_0070202</t>
+  </si>
+  <si>
+    <t>CAND_0006557</t>
   </si>
   <si>
     <t>CAND_0037980</t>
   </si>
   <si>
-    <t>CAND_0095528</t>
-  </si>
-  <si>
-    <t>CAND_0006557</t>
-  </si>
-  <si>
-    <t>CAND_0070202</t>
+    <t>CAND_0099401</t>
+  </si>
+  <si>
+    <t>CAND_0018722</t>
+  </si>
+  <si>
+    <t>CAND_0055992</t>
   </si>
   <si>
     <t>CAND_0052335</t>
   </si>
   <si>
-    <t>CAND_0099401</t>
-  </si>
-  <si>
-    <t>CAND_0018722</t>
-  </si>
-  <si>
     <t>CAND_0087630</t>
   </si>
   <si>
-    <t>CAND_0055992</t>
-  </si>
-  <si>
     <t>CAND_0033861</t>
   </si>
   <si>
+    <t>CAND_0015528</t>
+  </si>
+  <si>
+    <t>CAND_0013536</t>
+  </si>
+  <si>
     <t>CAND_0007412</t>
   </si>
   <si>
-    <t>CAND_0015528</t>
-  </si>
-  <si>
-    <t>CAND_0013536</t>
+    <t>CAND_0076163</t>
   </si>
   <si>
     <t>CAND_0072660</t>
   </si>
   <si>
-    <t>CAND_0076163</t>
-  </si>
-  <si>
     <t>CAND_0061257</t>
   </si>
   <si>
     <t>CAND_0094759</t>
   </si>
   <si>
+    <t>CAND_0067866</t>
+  </si>
+  <si>
+    <t>CAND_0068932</t>
+  </si>
+  <si>
+    <t>CAND_0069638</t>
+  </si>
+  <si>
+    <t>CAND_0093193</t>
+  </si>
+  <si>
     <t>CAND_0053605</t>
   </si>
   <si>
+    <t>CAND_0096104</t>
+  </si>
+  <si>
+    <t>CAND_0033179</t>
+  </si>
+  <si>
+    <t>CAND_0005509</t>
+  </si>
+  <si>
+    <t>CAND_0095619</t>
+  </si>
+  <si>
+    <t>CAND_0004402</t>
+  </si>
+  <si>
+    <t>CAND_0043860</t>
+  </si>
+  <si>
+    <t>CAND_0073007</t>
+  </si>
+  <si>
     <t>CAND_0048558</t>
   </si>
   <si>
-    <t>CAND_0093193</t>
-  </si>
-  <si>
-    <t>CAND_0067866</t>
-  </si>
-  <si>
-    <t>CAND_0005509</t>
+    <t>CAND_0046132</t>
+  </si>
+  <si>
+    <t>CAND_0070525</t>
   </si>
   <si>
     <t>CAND_0092278</t>
   </si>
   <si>
-    <t>CAND_0069638</t>
-  </si>
-  <si>
-    <t>CAND_0068932</t>
+    <t>CAND_0025882</t>
+  </si>
+  <si>
+    <t>CAND_0037160</t>
+  </si>
+  <si>
+    <t>CAND_0008295</t>
+  </si>
+  <si>
+    <t>CAND_0066035</t>
+  </si>
+  <si>
+    <t>CAND_0092255</t>
   </si>
   <si>
     <t>CAND_0052195</t>
   </si>
   <si>
-    <t>CAND_0095619</t>
-  </si>
-  <si>
-    <t>CAND_0004402</t>
-  </si>
-  <si>
-    <t>CAND_0096104</t>
-  </si>
-  <si>
-    <t>CAND_0043860</t>
-  </si>
-  <si>
-    <t>CAND_0092255</t>
-  </si>
-  <si>
-    <t>CAND_0073007</t>
-  </si>
-  <si>
-    <t>CAND_0033179</t>
-  </si>
-  <si>
-    <t>CAND_0025882</t>
-  </si>
-  <si>
-    <t>CAND_0070525</t>
-  </si>
-  <si>
     <t>CAND_0091745</t>
   </si>
   <si>
-    <t>CAND_0037160</t>
-  </si>
-  <si>
-    <t>CAND_0046132</t>
-  </si>
-  <si>
-    <t>CAND_0066035</t>
-  </si>
-  <si>
-    <t>CAND_0010149</t>
-  </si>
-  <si>
-    <t>CAND_0047327</t>
+    <t>CAND_0025640</t>
+  </si>
+  <si>
+    <t>CAND_0000273</t>
   </si>
   <si>
     <t>CAND_0032271</t>
   </si>
   <si>
-    <t>CAND_0068012</t>
-  </si>
-  <si>
-    <t>CAND_0026716</t>
-  </si>
-  <si>
-    <t>CAND_0017178</t>
-  </si>
-  <si>
-    <t>CAND_0067535</t>
-  </si>
-  <si>
-    <t>CAND_0097176</t>
+    <t>CAND_0026362</t>
+  </si>
+  <si>
+    <t>CAND_0092706</t>
+  </si>
+  <si>
+    <t>CAND_0046924</t>
+  </si>
+  <si>
+    <t>CAND_0035879</t>
   </si>
   <si>
     <t>Senior Machine Learning Engineer with 7.2 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in a preferred hub (Pune/Noida); response rate 61%).</t>
@@ -340,16 +340,19 @@
     <t>Senior Applied Scientist with 16.2 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, willing to relocate; response rate 81%).</t>
   </si>
   <si>
+    <t>AI Engineer with 6.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Strong JD fit (Tier-1 India city; response rate 77%).</t>
+  </si>
+  <si>
     <t>Senior NLP Engineer with 8.9 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 78%).</t>
   </si>
   <si>
-    <t>AI Engineer with 6.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Strong JD fit (Tier-1 India city; response rate 77%).</t>
+    <t>AI Engineer with 7.7 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 60%).</t>
   </si>
   <si>
     <t>Recommendation Systems Engineer with 7.7 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 72%).</t>
   </si>
   <si>
-    <t>AI Engineer with 7.7 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 60%).</t>
+    <t>Search Engineer with 7.6 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Strong JD fit (Tier-1 India city; response rate 94%).</t>
   </si>
   <si>
     <t>Senior NLP Engineer with 7.8 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 89%).</t>
@@ -358,21 +361,18 @@
     <t>NLP Engineer with 6.7 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 83%).</t>
   </si>
   <si>
-    <t>Search Engineer with 7.6 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Strong JD fit (Tier-1 India city; response rate 94%).</t>
+    <t>AI Engineer with 16.6 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 84%).</t>
   </si>
   <si>
     <t>Applied ML Engineer with 8.0 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Strong JD fit (in a preferred hub (Pune/Noida); response rate 42%).</t>
   </si>
   <si>
+    <t>Applied ML Engineer with 6.8 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 41%).</t>
+  </si>
+  <si>
     <t>Recommendation Systems Engineer with 7.9 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in a preferred hub (Pune/Noida); response rate 62%).</t>
   </si>
   <si>
-    <t>AI Engineer with 16.6 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 84%).</t>
-  </si>
-  <si>
-    <t>Applied ML Engineer with 6.8 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (Tier-1 India city; response rate 41%).</t>
-  </si>
-  <si>
     <t>Staff Machine Learning Engineer with 8.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong fit overall, though 90-day notice period; in India, relocation unclear.</t>
   </si>
   <si>
@@ -382,12 +382,12 @@
     <t>Senior AI Engineer with 7.8 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 76%).</t>
   </si>
   <si>
+    <t>AI Engineer with 6.9 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 81%).</t>
+  </si>
+  <si>
     <t>Senior NLP Engineer with 7.8 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong fit overall, though 90-day notice period; Tier-1 India city.</t>
   </si>
   <si>
-    <t>AI Engineer with 6.9 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Strong JD fit (in India, relocation unclear; response rate 81%).</t>
-  </si>
-  <si>
     <t>Senior Machine Learning Engineer with 8.1 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD).</t>
   </si>
   <si>
@@ -403,229 +403,229 @@
     <t>Senior Data Scientist with 7.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 90-day notice period.</t>
   </si>
   <si>
+    <t>Search Engineer with 7.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer with 7.2 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer with 6.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 90-day notice period.</t>
+  </si>
+  <si>
+    <t>Search Engineer with 7.2 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Recommendation Systems Engineer with 6.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer with 6.2 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
+  </si>
+  <si>
     <t>Applied ML Engineer with 7.1 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 90-day notice period.</t>
   </si>
   <si>
-    <t>Applied ML Engineer with 6.2 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Machine Learning Engineer with 7.2 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Applied ML Engineer with 6.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 90-day notice period.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.2 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Recommendation Systems Engineer with 6.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 120-day notice period.</t>
+    <t>Search Engineer with 7.6 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
+  </si>
+  <si>
+    <t>Search Engineer with 7.3 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 90-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist with 7.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer with 6.6 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
+  </si>
+  <si>
+    <t>Recommendation Systems Engineer with 7.7 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Recommendation Systems Engineer with 6.8 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
+  </si>
+  <si>
+    <t>AI Engineer with 7.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist with 5.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
+  </si>
+  <si>
+    <t>Recommendation Systems Engineer with 6.4 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
+  </si>
+  <si>
+    <t>Senior AI Engineer with 7.9 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; in a preferred hub (Pune/Noida).</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer with 6.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
+  </si>
+  <si>
+    <t>Search Engineer with 7.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 90-day notice period.</t>
   </si>
   <si>
     <t>NLP Engineer with 7.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 120-day notice period.</t>
   </si>
   <si>
-    <t>Senior Data Scientist with 7.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
-  </si>
-  <si>
-    <t>Recommendation Systems Engineer with 7.7 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.3 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 90-day notice period.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.6 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
-  </si>
-  <si>
-    <t>Recommendation Systems Engineer with 6.8 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
-  </si>
-  <si>
-    <t>Applied ML Engineer with 6.6 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
-  </si>
-  <si>
     <t>Senior Data Scientist with 6.5 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; in a preferred hub (Pune/Noida), but 120-day notice period.</t>
   </si>
   <si>
+    <t>Search Engineer with 6.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 120-day notice period.</t>
+  </si>
+  <si>
     <t>Applied ML Engineer with 6.7 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 120-day notice period.</t>
   </si>
   <si>
-    <t>AI Engineer with 7.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
-  </si>
-  <si>
-    <t>Senior Data Scientist with 5.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
-  </si>
-  <si>
-    <t>Senior AI Engineer with 7.9 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; in a preferred hub (Pune/Noida).</t>
-  </si>
-  <si>
-    <t>Machine Learning Engineer with 6.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
-  </si>
-  <si>
-    <t>Recommendation Systems Engineer with 6.4 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.8 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but 90-day notice period.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 6.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 120-day notice period.</t>
+    <t>AI Engineer with 5.3 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD).</t>
   </si>
   <si>
     <t>Recommendation Systems Engineer with 15.2 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but frequent short stints.</t>
   </si>
   <si>
-    <t>AI Engineer with 5.3 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD).</t>
+    <t>Senior Data Scientist with 7.8 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
+  </si>
+  <si>
+    <t>Search Engineer with 7.8 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but frequent short stints.</t>
   </si>
   <si>
     <t>NLP Engineer with 16.1 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; in India, willing to relocate.</t>
   </si>
   <si>
-    <t>Senior Data Scientist with 7.8 yrs, with documented embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
-  </si>
-  <si>
-    <t>Search Engineer with 7.8 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; Tier-1 India city, but frequent short stints.</t>
+    <t>Senior Data Scientist with 5.3 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer with 5.1 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 90-day notice period.</t>
+  </si>
+  <si>
+    <t>NLP Engineer with 7.9 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
   </si>
   <si>
     <t>Senior Applied Scientist with 9.0 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Solid match on the JD's retrieval/ranking core; Tier-1 India city.</t>
   </si>
   <si>
-    <t>Senior Data Scientist with 5.3 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear.</t>
-  </si>
-  <si>
-    <t>NLP Engineer with 7.9 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Machine Learning Engineer with 5.1 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, relocation unclear, but 90-day notice period.</t>
-  </si>
-  <si>
-    <t>Applied ML Engineer with 6.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD).</t>
-  </si>
-  <si>
     <t>NLP Engineer with 7.7 yrs; career history evidences embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Solid match on the JD's retrieval/ranking core; in India, willing to relocate, but 90-day notice period.</t>
   </si>
   <si>
     <t>Recommendation Systems Engineer with 6.6 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD), but 90-day notice period.</t>
   </si>
   <si>
+    <t>AI Engineer with 16.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Solid match on the JD's retrieval/ranking core; outside India (case-by-case per JD).</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer with 6.4 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Included toward the cutoff: outside India (case-by-case per JD); weaker depth than higher ranks.</t>
+  </si>
+  <si>
     <t>AI Engineer with 7.2 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
   </si>
   <si>
-    <t>AI Engineer with 16.9 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Included toward the cutoff: outside India (case-by-case per JD); weaker depth than higher ranks.</t>
-  </si>
-  <si>
     <t>Senior NLP Engineer with 8.0 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Included toward the cutoff: in India, relocation unclear; concerns — inactive ~115d on platform and low recruiter response rate (16%).</t>
   </si>
   <si>
+    <t>Applied ML Engineer with 7.4 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer with 14.1 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: in India, relocation unclear; concerns — 90-day notice period.</t>
+  </si>
+  <si>
     <t>Applied ML Engineer with 7.4 yrs; career history evidences embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); concerns — 120-day notice period and frequent short stints.</t>
   </si>
   <si>
-    <t>Applied ML Engineer with 7.4 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Applied ML Engineer with 14.1 yrs — demonstrated embeddings/retrieval work, shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: in India, relocation unclear; concerns — 90-day notice period.</t>
+    <t>NLP Engineer with 6.9 yrs; career history evidences shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
   </si>
   <si>
     <t>Machine Learning Engineer with 7.1 yrs — demonstrated embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems in past roles. Included toward the cutoff: outside India (case-by-case per JD); weaker depth than higher ranks.</t>
   </si>
   <si>
-    <t>NLP Engineer with 6.9 yrs; career history evidences shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style). Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
-  </si>
-  <si>
     <t>Staff Machine Learning Engineer with 8.0 yrs — demonstrated embeddings/retrieval work and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
   </si>
   <si>
     <t>Lead AI Engineer with 8.6 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; concerns — inactive ~154d on platform and low recruiter response rate (11%).</t>
   </si>
   <si>
+    <t>Senior Software Engineer (ML) with 6.4 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>ML Engineer with 5.2 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Computer Vision Engineer with 6.2 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer with 7.9 yrs, with documented embeddings/retrieval work and ranking-evaluation rigor (NDCG/MRR/A-B style). Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
     <t>Senior Software Engineer (ML) with 6.9 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
   </si>
   <si>
+    <t>AI Specialist with 7.0 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer with 6.9 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in India, willing to relocate; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Data Scientist with 6.0 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>NLP Engineer with 15.6 yrs — demonstrated shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer with 6.0 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Junior ML Engineer with 6.1 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: in India, willing to relocate; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>AI Specialist with 5.8 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
     <t>Data Scientist with 6.7 yrs — demonstrated shipped ranking/recommendation systems in past roles. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
   </si>
   <si>
-    <t>Senior Machine Learning Engineer with 7.9 yrs, with documented embeddings/retrieval work and ranking-evaluation rigor (NDCG/MRR/A-B style). Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Senior Software Engineer (ML) with 6.4 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Data Scientist with 6.0 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+    <t>AI Research Engineer with 4.3 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) with 5.4 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
   </si>
   <si>
     <t>Senior NLP Engineer with 6.8 yrs, with documented embeddings/retrieval work, vector/hybrid search infrastructure and shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); concerns — inactive ~216d on platform and low recruiter response rate (7%).</t>
   </si>
   <si>
-    <t>Computer Vision Engineer with 6.2 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>ML Engineer with 5.2 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+    <t>Senior Software Engineer (ML) with 5.6 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Data Scientist with 6.0 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer with 6.5 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>Data Scientist with 6.7 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>ML Engineer with 5.2 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
   </si>
   <si>
     <t>Computer Vision Engineer with 6.3 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
   </si>
   <si>
-    <t>NLP Engineer with 15.6 yrs — demonstrated shipped ranking/recommendation systems and ranking-evaluation rigor (NDCG/MRR/A-B style) in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>AI Research Engineer with 6.0 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>AI Specialist with 7.0 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Junior ML Engineer with 6.1 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: in India, willing to relocate; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>ML Engineer with 5.2 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>AI Specialist with 5.8 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>AI Research Engineer with 6.9 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in India, willing to relocate; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Senior Software Engineer (ML) with 5.6 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Senior Software Engineer (ML) with 5.4 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
     <t>Junior ML Engineer with 5.9 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
   </si>
   <si>
-    <t>Data Scientist with 6.0 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>AI Research Engineer with 4.3 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Data Scientist with 6.7 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>ML Engineer with 6.9 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: Tier-1 India city; concerns — 90-day notice period.</t>
-  </si>
-  <si>
-    <t>Junior ML Engineer with 5.0 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+    <t>AI Research Engineer with 5.6 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>ML Engineer with 5.8 yrs — demonstrated shipped ranking/recommendation systems in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
   </si>
   <si>
     <t>AI Research Engineer with 6.6 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: Tier-1 India city; concerns — 120-day notice period.</t>
   </si>
   <si>
-    <t>Junior ML Engineer with 5.7 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); concerns — 120-day notice period.</t>
-  </si>
-  <si>
-    <t>Computer Vision Engineer with 5.6 yrs, with documented shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in India, willing to relocate; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>ML Engineer with 4.2 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>Junior ML Engineer with 6.8 yrs; career history evidences shipped ranking/recommendation systems and LLM/fine-tuning exposure. Included toward the cutoff: in India, relocation unclear; weaker depth than higher ranks.</t>
-  </si>
-  <si>
-    <t>ML Engineer with 5.9 yrs — demonstrated shipped ranking/recommendation systems and LLM/fine-tuning exposure in past roles. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+    <t>Data Scientist with 5.0 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: Tier-1 India city; weaker depth than higher ranks.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer with 5.8 yrs — demonstrated shipped ranking/recommendation systems in past roles. Included toward the cutoff: Tier-1 India city; concerns — 120-day notice period.</t>
+  </si>
+  <si>
+    <t>Computer Vision Engineer with 6.3 yrs, with documented shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); concerns — 120-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer with 4.5 yrs; career history evidences shipped ranking/recommendation systems. Included toward the cutoff: in a preferred hub (Pune/Noida); concerns — 120-day notice period.</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1008,7 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.985791</v>
+        <v>1.030756</v>
       </c>
       <c r="D2" t="s">
         <v>104</v>
@@ -1022,7 +1022,7 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.9463009999999999</v>
+        <v>0.999455</v>
       </c>
       <c r="D3" t="s">
         <v>105</v>
@@ -1036,7 +1036,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>0.897482</v>
+        <v>0.945242</v>
       </c>
       <c r="D4" t="s">
         <v>106</v>
@@ -1050,7 +1050,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>0.89573</v>
+        <v>0.9401119999999999</v>
       </c>
       <c r="D5" t="s">
         <v>107</v>
@@ -1064,7 +1064,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>0.867802</v>
+        <v>0.917631</v>
       </c>
       <c r="D6" t="s">
         <v>108</v>
@@ -1078,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>0.855772</v>
+        <v>0.90606</v>
       </c>
       <c r="D7" t="s">
         <v>109</v>
@@ -1092,7 +1092,7 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>0.841575</v>
+        <v>0.894581</v>
       </c>
       <c r="D8" t="s">
         <v>110</v>
@@ -1106,7 +1106,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.826954</v>
+        <v>0.891149</v>
       </c>
       <c r="D9" t="s">
         <v>111</v>
@@ -1120,7 +1120,7 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <v>0.816844</v>
+        <v>0.866706</v>
       </c>
       <c r="D10" t="s">
         <v>112</v>
@@ -1134,7 +1134,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.808833</v>
+        <v>0.8618749999999999</v>
       </c>
       <c r="D11" t="s">
         <v>113</v>
@@ -1148,7 +1148,7 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>0.801919</v>
+        <v>0.859232</v>
       </c>
       <c r="D12" t="s">
         <v>114</v>
@@ -1162,7 +1162,7 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>0.799966</v>
+        <v>0.858199</v>
       </c>
       <c r="D13" t="s">
         <v>115</v>
@@ -1176,7 +1176,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>0.798822</v>
+        <v>0.853426</v>
       </c>
       <c r="D14" t="s">
         <v>116</v>
@@ -1190,7 +1190,7 @@
         <v>14</v>
       </c>
       <c r="C15">
-        <v>0.798173</v>
+        <v>0.845166</v>
       </c>
       <c r="D15" t="s">
         <v>117</v>
@@ -1204,7 +1204,7 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>0.795719</v>
+        <v>0.842615</v>
       </c>
       <c r="D16" t="s">
         <v>118</v>
@@ -1218,7 +1218,7 @@
         <v>16</v>
       </c>
       <c r="C17">
-        <v>0.783017</v>
+        <v>0.836241</v>
       </c>
       <c r="D17" t="s">
         <v>119</v>
@@ -1232,7 +1232,7 @@
         <v>17</v>
       </c>
       <c r="C18">
-        <v>0.765293</v>
+        <v>0.833281</v>
       </c>
       <c r="D18" t="s">
         <v>120</v>
@@ -1246,7 +1246,7 @@
         <v>18</v>
       </c>
       <c r="C19">
-        <v>0.764341</v>
+        <v>0.814823</v>
       </c>
       <c r="D19" t="s">
         <v>121</v>
@@ -1260,7 +1260,7 @@
         <v>19</v>
       </c>
       <c r="C20">
-        <v>0.7587</v>
+        <v>0.805725</v>
       </c>
       <c r="D20" t="s">
         <v>122</v>
@@ -1274,7 +1274,7 @@
         <v>20</v>
       </c>
       <c r="C21">
-        <v>0.7537509999999999</v>
+        <v>0.797982</v>
       </c>
       <c r="D21" t="s">
         <v>123</v>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C22">
-        <v>0.7519749999999999</v>
+        <v>0.797138</v>
       </c>
       <c r="D22" t="s">
         <v>124</v>
@@ -1302,7 +1302,7 @@
         <v>22</v>
       </c>
       <c r="C23">
-        <v>0.742642</v>
+        <v>0.788901</v>
       </c>
       <c r="D23" t="s">
         <v>125</v>
@@ -1316,7 +1316,7 @@
         <v>23</v>
       </c>
       <c r="C24">
-        <v>0.72682</v>
+        <v>0.787889</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -1330,7 +1330,7 @@
         <v>24</v>
       </c>
       <c r="C25">
-        <v>0.718904</v>
+        <v>0.7700709999999999</v>
       </c>
       <c r="D25" t="s">
         <v>127</v>
@@ -1344,7 +1344,7 @@
         <v>25</v>
       </c>
       <c r="C26">
-        <v>0.705426</v>
+        <v>0.762092</v>
       </c>
       <c r="D26" t="s">
         <v>128</v>
@@ -1358,7 +1358,7 @@
         <v>26</v>
       </c>
       <c r="C27">
-        <v>0.704268</v>
+        <v>0.759557</v>
       </c>
       <c r="D27" t="s">
         <v>129</v>
@@ -1372,7 +1372,7 @@
         <v>27</v>
       </c>
       <c r="C28">
-        <v>0.702352</v>
+        <v>0.758433</v>
       </c>
       <c r="D28" t="s">
         <v>130</v>
@@ -1386,7 +1386,7 @@
         <v>28</v>
       </c>
       <c r="C29">
-        <v>0.697819</v>
+        <v>0.755861</v>
       </c>
       <c r="D29" t="s">
         <v>131</v>
@@ -1400,7 +1400,7 @@
         <v>29</v>
       </c>
       <c r="C30">
-        <v>0.697805</v>
+        <v>0.755119</v>
       </c>
       <c r="D30" t="s">
         <v>132</v>
@@ -1414,7 +1414,7 @@
         <v>30</v>
       </c>
       <c r="C31">
-        <v>0.695311</v>
+        <v>0.755014</v>
       </c>
       <c r="D31" t="s">
         <v>133</v>
@@ -1428,7 +1428,7 @@
         <v>31</v>
       </c>
       <c r="C32">
-        <v>0.6911310000000001</v>
+        <v>0.75479</v>
       </c>
       <c r="D32" t="s">
         <v>134</v>
@@ -1442,7 +1442,7 @@
         <v>32</v>
       </c>
       <c r="C33">
-        <v>0.688972</v>
+        <v>0.749245</v>
       </c>
       <c r="D33" t="s">
         <v>135</v>
@@ -1456,7 +1456,7 @@
         <v>33</v>
       </c>
       <c r="C34">
-        <v>0.677616</v>
+        <v>0.737277</v>
       </c>
       <c r="D34" t="s">
         <v>136</v>
@@ -1470,7 +1470,7 @@
         <v>34</v>
       </c>
       <c r="C35">
-        <v>0.671686</v>
+        <v>0.735241</v>
       </c>
       <c r="D35" t="s">
         <v>137</v>
@@ -1484,7 +1484,7 @@
         <v>35</v>
       </c>
       <c r="C36">
-        <v>0.670243</v>
+        <v>0.726535</v>
       </c>
       <c r="D36" t="s">
         <v>138</v>
@@ -1498,7 +1498,7 @@
         <v>36</v>
       </c>
       <c r="C37">
-        <v>0.665691</v>
+        <v>0.723442</v>
       </c>
       <c r="D37" t="s">
         <v>139</v>
@@ -1512,7 +1512,7 @@
         <v>37</v>
       </c>
       <c r="C38">
-        <v>0.664289</v>
+        <v>0.722012</v>
       </c>
       <c r="D38" t="s">
         <v>140</v>
@@ -1526,7 +1526,7 @@
         <v>38</v>
       </c>
       <c r="C39">
-        <v>0.660048</v>
+        <v>0.719307</v>
       </c>
       <c r="D39" t="s">
         <v>141</v>
@@ -1540,7 +1540,7 @@
         <v>39</v>
       </c>
       <c r="C40">
-        <v>0.659906</v>
+        <v>0.718639</v>
       </c>
       <c r="D40" t="s">
         <v>142</v>
@@ -1554,7 +1554,7 @@
         <v>40</v>
       </c>
       <c r="C41">
-        <v>0.655774</v>
+        <v>0.710171</v>
       </c>
       <c r="D41" t="s">
         <v>143</v>
@@ -1568,7 +1568,7 @@
         <v>41</v>
       </c>
       <c r="C42">
-        <v>0.653026</v>
+        <v>0.704684</v>
       </c>
       <c r="D42" t="s">
         <v>144</v>
@@ -1582,7 +1582,7 @@
         <v>42</v>
       </c>
       <c r="C43">
-        <v>0.649002</v>
+        <v>0.698581</v>
       </c>
       <c r="D43" t="s">
         <v>145</v>
@@ -1596,7 +1596,7 @@
         <v>43</v>
       </c>
       <c r="C44">
-        <v>0.645723</v>
+        <v>0.697932</v>
       </c>
       <c r="D44" t="s">
         <v>146</v>
@@ -1610,7 +1610,7 @@
         <v>44</v>
       </c>
       <c r="C45">
-        <v>0.643456</v>
+        <v>0.693068</v>
       </c>
       <c r="D45" t="s">
         <v>147</v>
@@ -1624,7 +1624,7 @@
         <v>45</v>
       </c>
       <c r="C46">
-        <v>0.638958</v>
+        <v>0.693057</v>
       </c>
       <c r="D46" t="s">
         <v>148</v>
@@ -1638,7 +1638,7 @@
         <v>46</v>
       </c>
       <c r="C47">
-        <v>0.637503</v>
+        <v>0.691294</v>
       </c>
       <c r="D47" t="s">
         <v>149</v>
@@ -1652,7 +1652,7 @@
         <v>47</v>
       </c>
       <c r="C48">
-        <v>0.630474</v>
+        <v>0.689714</v>
       </c>
       <c r="D48" t="s">
         <v>150</v>
@@ -1666,7 +1666,7 @@
         <v>48</v>
       </c>
       <c r="C49">
-        <v>0.629753</v>
+        <v>0.681889</v>
       </c>
       <c r="D49" t="s">
         <v>151</v>
@@ -1680,7 +1680,7 @@
         <v>49</v>
       </c>
       <c r="C50">
-        <v>0.6270829999999999</v>
+        <v>0.679579</v>
       </c>
       <c r="D50" t="s">
         <v>152</v>
@@ -1694,7 +1694,7 @@
         <v>50</v>
       </c>
       <c r="C51">
-        <v>0.625528</v>
+        <v>0.663394</v>
       </c>
       <c r="D51" t="s">
         <v>153</v>
@@ -1708,7 +1708,7 @@
         <v>51</v>
       </c>
       <c r="C52">
-        <v>0.619539</v>
+        <v>0.647529</v>
       </c>
       <c r="D52" t="s">
         <v>154</v>
@@ -1722,7 +1722,7 @@
         <v>52</v>
       </c>
       <c r="C53">
-        <v>0.590184</v>
+        <v>0.6457889999999999</v>
       </c>
       <c r="D53" t="s">
         <v>155</v>
@@ -1736,7 +1736,7 @@
         <v>53</v>
       </c>
       <c r="C54">
-        <v>0.58853</v>
+        <v>0.64469</v>
       </c>
       <c r="D54" t="s">
         <v>156</v>
@@ -1750,7 +1750,7 @@
         <v>54</v>
       </c>
       <c r="C55">
-        <v>0.579103</v>
+        <v>0.628789</v>
       </c>
       <c r="D55" t="s">
         <v>157</v>
@@ -1764,7 +1764,7 @@
         <v>55</v>
       </c>
       <c r="C56">
-        <v>0.570753</v>
+        <v>0.628682</v>
       </c>
       <c r="D56" t="s">
         <v>158</v>
@@ -1778,7 +1778,7 @@
         <v>56</v>
       </c>
       <c r="C57">
-        <v>0.568519</v>
+        <v>0.6272450000000001</v>
       </c>
       <c r="D57" t="s">
         <v>159</v>
@@ -1792,7 +1792,7 @@
         <v>57</v>
       </c>
       <c r="C58">
-        <v>0.566111</v>
+        <v>0.6254999999999999</v>
       </c>
       <c r="D58" t="s">
         <v>160</v>
@@ -1806,7 +1806,7 @@
         <v>58</v>
       </c>
       <c r="C59">
-        <v>0.565019</v>
+        <v>0.619003</v>
       </c>
       <c r="D59" t="s">
         <v>161</v>
@@ -1820,7 +1820,7 @@
         <v>59</v>
       </c>
       <c r="C60">
-        <v>0.562389</v>
+        <v>0.617112</v>
       </c>
       <c r="D60" t="s">
         <v>162</v>
@@ -1834,7 +1834,7 @@
         <v>60</v>
       </c>
       <c r="C61">
-        <v>0.551267</v>
+        <v>0.6155040000000001</v>
       </c>
       <c r="D61" t="s">
         <v>163</v>
@@ -1848,7 +1848,7 @@
         <v>61</v>
       </c>
       <c r="C62">
-        <v>0.550534</v>
+        <v>0.614128</v>
       </c>
       <c r="D62" t="s">
         <v>164</v>
@@ -1862,7 +1862,7 @@
         <v>62</v>
       </c>
       <c r="C63">
-        <v>0.550041</v>
+        <v>0.606401</v>
       </c>
       <c r="D63" t="s">
         <v>165</v>
@@ -1876,7 +1876,7 @@
         <v>63</v>
       </c>
       <c r="C64">
-        <v>0.542856</v>
+        <v>0.578496</v>
       </c>
       <c r="D64" t="s">
         <v>166</v>
@@ -1890,7 +1890,7 @@
         <v>64</v>
       </c>
       <c r="C65">
-        <v>0.515185</v>
+        <v>0.572106</v>
       </c>
       <c r="D65" t="s">
         <v>167</v>
@@ -1904,7 +1904,7 @@
         <v>65</v>
       </c>
       <c r="C66">
-        <v>0.512603</v>
+        <v>0.561517</v>
       </c>
       <c r="D66" t="s">
         <v>168</v>
@@ -1918,7 +1918,7 @@
         <v>66</v>
       </c>
       <c r="C67">
-        <v>0.500955</v>
+        <v>0.556871</v>
       </c>
       <c r="D67" t="s">
         <v>169</v>
@@ -1932,7 +1932,7 @@
         <v>67</v>
       </c>
       <c r="C68">
-        <v>0.496092</v>
+        <v>0.53459</v>
       </c>
       <c r="D68" t="s">
         <v>170</v>
@@ -1946,7 +1946,7 @@
         <v>68</v>
       </c>
       <c r="C69">
-        <v>0.480093</v>
+        <v>0.532702</v>
       </c>
       <c r="D69" t="s">
         <v>171</v>
@@ -1960,7 +1960,7 @@
         <v>69</v>
       </c>
       <c r="C70">
-        <v>0.477427</v>
+        <v>0.5241440000000001</v>
       </c>
       <c r="D70" t="s">
         <v>172</v>
@@ -1974,7 +1974,7 @@
         <v>70</v>
       </c>
       <c r="C71">
-        <v>0.465371</v>
+        <v>0.502335</v>
       </c>
       <c r="D71" t="s">
         <v>173</v>
@@ -1988,7 +1988,7 @@
         <v>71</v>
       </c>
       <c r="C72">
-        <v>0.429731</v>
+        <v>0.475559</v>
       </c>
       <c r="D72" t="s">
         <v>174</v>
@@ -2002,7 +2002,7 @@
         <v>72</v>
       </c>
       <c r="C73">
-        <v>0.428626</v>
+        <v>0.474401</v>
       </c>
       <c r="D73" t="s">
         <v>175</v>
@@ -2016,7 +2016,7 @@
         <v>73</v>
       </c>
       <c r="C74">
-        <v>0.425052</v>
+        <v>0.473496</v>
       </c>
       <c r="D74" t="s">
         <v>176</v>
@@ -2030,7 +2030,7 @@
         <v>74</v>
       </c>
       <c r="C75">
-        <v>0.42454</v>
+        <v>0.472405</v>
       </c>
       <c r="D75" t="s">
         <v>177</v>
@@ -2044,7 +2044,7 @@
         <v>75</v>
       </c>
       <c r="C76">
-        <v>0.422852</v>
+        <v>0.470566</v>
       </c>
       <c r="D76" t="s">
         <v>178</v>
@@ -2058,7 +2058,7 @@
         <v>76</v>
       </c>
       <c r="C77">
-        <v>0.419535</v>
+        <v>0.469624</v>
       </c>
       <c r="D77" t="s">
         <v>179</v>
@@ -2072,7 +2072,7 @@
         <v>77</v>
       </c>
       <c r="C78">
-        <v>0.416584</v>
+        <v>0.466085</v>
       </c>
       <c r="D78" t="s">
         <v>180</v>
@@ -2086,7 +2086,7 @@
         <v>78</v>
       </c>
       <c r="C79">
-        <v>0.416402</v>
+        <v>0.465643</v>
       </c>
       <c r="D79" t="s">
         <v>181</v>
@@ -2100,7 +2100,7 @@
         <v>79</v>
       </c>
       <c r="C80">
-        <v>0.415987</v>
+        <v>0.464664</v>
       </c>
       <c r="D80" t="s">
         <v>182</v>
@@ -2114,7 +2114,7 @@
         <v>80</v>
       </c>
       <c r="C81">
-        <v>0.408973</v>
+        <v>0.462459</v>
       </c>
       <c r="D81" t="s">
         <v>183</v>
@@ -2128,7 +2128,7 @@
         <v>81</v>
       </c>
       <c r="C82">
-        <v>0.407379</v>
+        <v>0.459316</v>
       </c>
       <c r="D82" t="s">
         <v>184</v>
@@ -2142,7 +2142,7 @@
         <v>82</v>
       </c>
       <c r="C83">
-        <v>0.404266</v>
+        <v>0.458476</v>
       </c>
       <c r="D83" t="s">
         <v>185</v>
@@ -2156,7 +2156,7 @@
         <v>83</v>
       </c>
       <c r="C84">
-        <v>0.403955</v>
+        <v>0.457758</v>
       </c>
       <c r="D84" t="s">
         <v>186</v>
@@ -2170,7 +2170,7 @@
         <v>84</v>
       </c>
       <c r="C85">
-        <v>0.401854</v>
+        <v>0.449803</v>
       </c>
       <c r="D85" t="s">
         <v>187</v>
@@ -2184,7 +2184,7 @@
         <v>85</v>
       </c>
       <c r="C86">
-        <v>0.400474</v>
+        <v>0.448524</v>
       </c>
       <c r="D86" t="s">
         <v>188</v>
@@ -2198,7 +2198,7 @@
         <v>86</v>
       </c>
       <c r="C87">
-        <v>0.399981</v>
+        <v>0.447889</v>
       </c>
       <c r="D87" t="s">
         <v>189</v>
@@ -2212,7 +2212,7 @@
         <v>87</v>
       </c>
       <c r="C88">
-        <v>0.396784</v>
+        <v>0.446289</v>
       </c>
       <c r="D88" t="s">
         <v>190</v>
@@ -2226,7 +2226,7 @@
         <v>88</v>
       </c>
       <c r="C89">
-        <v>0.394086</v>
+        <v>0.444556</v>
       </c>
       <c r="D89" t="s">
         <v>191</v>
@@ -2240,7 +2240,7 @@
         <v>89</v>
       </c>
       <c r="C90">
-        <v>0.390972</v>
+        <v>0.44195</v>
       </c>
       <c r="D90" t="s">
         <v>192</v>
@@ -2254,7 +2254,7 @@
         <v>90</v>
       </c>
       <c r="C91">
-        <v>0.390281</v>
+        <v>0.441329</v>
       </c>
       <c r="D91" t="s">
         <v>193</v>
@@ -2268,7 +2268,7 @@
         <v>91</v>
       </c>
       <c r="C92">
-        <v>0.383579</v>
+        <v>0.438976</v>
       </c>
       <c r="D92" t="s">
         <v>194</v>
@@ -2282,7 +2282,7 @@
         <v>92</v>
       </c>
       <c r="C93">
-        <v>0.381703</v>
+        <v>0.434344</v>
       </c>
       <c r="D93" t="s">
         <v>195</v>
@@ -2296,7 +2296,7 @@
         <v>93</v>
       </c>
       <c r="C94">
-        <v>0.380876</v>
+        <v>0.433669</v>
       </c>
       <c r="D94" t="s">
         <v>196</v>
@@ -2310,7 +2310,7 @@
         <v>94</v>
       </c>
       <c r="C95">
-        <v>0.380248</v>
+        <v>0.431336</v>
       </c>
       <c r="D95" t="s">
         <v>197</v>
@@ -2324,7 +2324,7 @@
         <v>95</v>
       </c>
       <c r="C96">
-        <v>0.380167</v>
+        <v>0.430569</v>
       </c>
       <c r="D96" t="s">
         <v>198</v>
@@ -2338,7 +2338,7 @@
         <v>96</v>
       </c>
       <c r="C97">
-        <v>0.377977</v>
+        <v>0.429771</v>
       </c>
       <c r="D97" t="s">
         <v>199</v>
@@ -2352,7 +2352,7 @@
         <v>97</v>
       </c>
       <c r="C98">
-        <v>0.375548</v>
+        <v>0.429681</v>
       </c>
       <c r="D98" t="s">
         <v>200</v>
@@ -2366,7 +2366,7 @@
         <v>98</v>
       </c>
       <c r="C99">
-        <v>0.375238</v>
+        <v>0.428867</v>
       </c>
       <c r="D99" t="s">
         <v>201</v>
@@ -2380,7 +2380,7 @@
         <v>99</v>
       </c>
       <c r="C100">
-        <v>0.374668</v>
+        <v>0.427274</v>
       </c>
       <c r="D100" t="s">
         <v>202</v>
@@ -2394,7 +2394,7 @@
         <v>100</v>
       </c>
       <c r="C101">
-        <v>0.373852</v>
+        <v>0.425364</v>
       </c>
       <c r="D101" t="s">
         <v>203</v>

</xml_diff>